<commit_message>
metida nota media clase E1A a excel primera evaluación
</commit_message>
<xml_diff>
--- a/matematicas_1ESOA/notas/E1A_eval1.xlsx
+++ b/matematicas_1ESOA/notas/E1A_eval1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\OneDrive\Desktop\sapere_aude\matematicas_1ESOA\notas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ac4744725179635e/Desktop/sapere_aude/matematicas_1ESOA/notas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFBE2993-C89A-4F1B-8212-DF3077A3A339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{FFBE2993-C89A-4F1B-8212-DF3077A3A339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46BC19A7-0762-4F93-9C86-CFEE21F23E85}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -656,7 +656,7 @@
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -791,6 +791,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Explanatory Text" xfId="2" builtinId="53" customBuiltin="1"/>
@@ -3577,6 +3578,10 @@
       </c>
       <c r="S28" s="33"/>
       <c r="T28" s="33"/>
+      <c r="U28" s="56">
+        <f>AVERAGE(U2:U26)</f>
+        <v>6.5082857142857131</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
parcial de probabilidad 2bach hecho. parcial de algebra 1eso en curso
</commit_message>
<xml_diff>
--- a/matematicas_1ESOA/notas/E1A_eval1.xlsx
+++ b/matematicas_1ESOA/notas/E1A_eval1.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">Actilla!$A$1:$Y$28</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -779,19 +779,19 @@
     <xf numFmtId="1" fontId="5" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Explanatory Text" xfId="2" builtinId="53" customBuiltin="1"/>
@@ -1417,16 +1417,16 @@
       </c>
     </row>
     <row r="8" spans="2:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="52" t="s">
+      <c r="B8" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
-      <c r="G8" s="52"/>
-      <c r="H8" s="52"/>
-      <c r="I8" s="52"/>
+      <c r="C8" s="56"/>
+      <c r="D8" s="56"/>
+      <c r="E8" s="56"/>
+      <c r="F8" s="56"/>
+      <c r="G8" s="56"/>
+      <c r="H8" s="56"/>
+      <c r="I8" s="56"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C9" s="2" t="s">
@@ -1444,16 +1444,16 @@
       </c>
     </row>
     <row r="15" spans="2:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="52" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="52"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="52"/>
-      <c r="F15" s="52"/>
-      <c r="G15" s="52"/>
-      <c r="H15" s="52"/>
-      <c r="I15" s="52"/>
+      <c r="B15" s="56" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="56"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="56"/>
+      <c r="G15" s="56"/>
+      <c r="H15" s="56"/>
+      <c r="I15" s="56"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
@@ -1476,16 +1476,16 @@
       </c>
     </row>
     <row r="22" spans="2:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="52" t="s">
+      <c r="B22" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="52"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="52"/>
-      <c r="H22" s="52"/>
-      <c r="I22" s="52"/>
+      <c r="C22" s="56"/>
+      <c r="D22" s="56"/>
+      <c r="E22" s="56"/>
+      <c r="F22" s="56"/>
+      <c r="G22" s="56"/>
+      <c r="H22" s="56"/>
+      <c r="I22" s="56"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.3">
       <c r="N23" s="4" t="s">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="S28" s="33"/>
       <c r="T28" s="33"/>
-      <c r="U28" s="56">
+      <c r="U28" s="52">
         <f>AVERAGE(U2:U26)</f>
         <v>6.5082857142857131</v>
       </c>

</xml_diff>